<commit_message>
Auto update P2P and organization activities 2026-04-21 18:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -428,27 +428,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Dia</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Sesión</t>
+          <t>Session</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mentor/a</t>
+          <t>Mentor/a Aula Nucli</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Comentario</t>
+          <t>Comentari</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Actividad</t>
+          <t>Activitat</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Alana)
+11:00 - De la Teoria a la Pràctica: Apps amb Streamlit</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
           <t>Alana</t>
@@ -1963,12 +1968,7 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Píldores Aula Nucli (Alana)
-11:00 - De la Teoria a la Pràctica: Apps amb Streamlit</t>
-        </is>
-      </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>Dago</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-04-22 13:25
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -550,8 +550,7 @@
         <is>
           <t>Presentacions
 11:00 - Francesco Eirado: Tendencias Globales y Desafíos Energéticos
-11:30 - Minu Campoy: Crecimiento, concentración y proyección en el tráfico aéreo de El Prat post-pandemia
-12:00 - Presentació Simulador: Verónica</t>
+11:30 - Minu Campoy: Crecimiento, concentración y proyección en el tráfico aéreo de El Prat post-pandemia</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -661,7 +660,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presentacions
+</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -763,7 +767,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Presentacions
+12:00 - Dioulde Diao: TBD</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-04-28 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -719,7 +719,11 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Best practices para crear una dashboard</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -1030,7 +1034,11 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Introducción a BIGQUERY </t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-04-30 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -721,7 +721,8 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Best practices para crear una dashboard</t>
+          <t>Píldora Aula Nucli
+11:00 - Taller de comunicación. Explorando la conciencia emocional y la comunicación no violenta para practicar cómo comunicarnos mejor y enfrentar conflictos en el contexto laboral.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1248,7 +1249,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Píldora Aula Nucli
+11:00 - Buenas prácticas para dashboards</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -1774,7 +1780,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Píldora Aula Nucli
+11:00 - Un caso real de projecto en Booking.com</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-05 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -722,7 +722,7 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Píldora Aula Nucli
-11:00 - Taller de comunicación. Explorando la conciencia emocional y la comunicación no violenta para practicar cómo comunicarnos mejor y enfrentar conflictos en el contexto laboral.</t>
+11:00 - 13:30 Taller de comunicación. Explorando la conciencia emocional y la comunicación no violenta para practicar cómo comunicarnos mejor y enfrentar conflictos en el contexto laboral y más allá. (Esto es un taller con prácticas en parejas y grupales, de una duración de dos horas y media, con una pequeña pausa en el medio.)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -775,7 +775,7 @@
       <c r="C13" t="inlineStr">
         <is>
           <t>Presentacions
-12:00 - Dioulde Diao: TBD</t>
+11:00 - Rocío Arias: TBD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -831,7 +831,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Alana)
+11:00 - De la Teoria a la Pràctica: Apps amb Streamlit</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>Alana</t>
@@ -879,7 +884,14 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Presentacions
+11:00 - Federico Urbina: TBD
+11:30 - Sabina Planas: TBD
+12:00 - Dioulde Diao: TBD</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>Joan</t>
@@ -981,7 +993,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Presentacions
+11:00 - Vanessa Bujaldon: TBD</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -1087,7 +1104,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Presentacions
+11:00 - Vanina Tonzo: TBD</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>Alana</t>
@@ -1358,20 +1380,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Píldores Aula Nucli (Alana)
-11:00 - Estructures de dades amb Python
-12:30 - Estructures de control amb Python</t>
+          <t>Dinàmiques Grupals:
+12:00 a 14:00 - Gestió de l'estrès en entorns d'alt rendiment 1</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Elixabete</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Píldoras</t>
+          <t>Otras Actividades</t>
         </is>
       </c>
     </row>
@@ -1386,18 +1407,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Irene</t>
+          <t>Dinàmiques Grupals:
+10:30 a 12:00 - Gestió de l'estrès en entorns d'alt rendiment 2</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Elixabete</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Tutoría de Proyectos</t>
+          <t>Otras Actividades</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1912,7 @@
       <c r="C55" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Alana)
-11:00 - De la Teoria a la Pràctica: Apps amb Streamlit</t>
+11:00 - Github en equipo: Básicos</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1965,6 +1987,108 @@
         </is>
       </c>
       <c r="C58" t="inlineStr">
+        <is>
+          <t>Welcome: de 10:15 – 11:00 
+Weekly: 
+11:00 Alana 
+12:00 Yunier 
+12:30 Dago 
+13:00 Irene
+Aquesta setmana el Joan està en remot</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Dago</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Alana</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Presentación de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -1975,98 +2099,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>46231</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr">
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Dago</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>46232</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Alana</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>46233</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr">
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>46272</v>
-      </c>
-      <c r="B62" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B66" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2077,98 +2201,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>46273</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr">
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Yunier</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>46274</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Dago</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>46275</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr">
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>46279</v>
-      </c>
-      <c r="B66" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B70" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2179,98 +2303,102 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>46280</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr">
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Joan</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Yunier</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Festivo</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>46282</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Dago</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="1" t="n">
-        <v>46286</v>
-      </c>
-      <c r="B70" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B74" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2281,102 +2409,110 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Dago</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Alana)
+Todo Python
+10:30 - Estructuras de datos
+11:30 - Estructuras de control
+12:30 - Funciones</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="1" t="n">
-        <v>46287</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr">
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Irene</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="1" t="n">
-        <v>46288</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Joan</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Festivo</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="1" t="n">
-        <v>46289</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Festivo</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr">
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="1" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B74" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B78" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2387,102 +2523,194 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr">
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Alana</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Presentación de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Festivo</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
         <is>
           <t>Welcome / Weekley</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="1" t="n">
-        <v>46294</v>
-      </c>
-      <c r="B75" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B83" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr">
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Dago</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Dago</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="1" t="n">
-        <v>46295</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Irene</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="1" t="n">
-        <v>46296</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Festivo</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr">
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="1" t="n">
-        <v>46300</v>
-      </c>
-      <c r="B78" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B86" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2493,194 +2721,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Yunier</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="1" t="n">
-        <v>46301</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr">
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="1" t="n">
-        <v>46302</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Alana</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="1" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr">
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="1" t="n">
-        <v>46307</v>
-      </c>
-      <c r="B82" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B90" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Festivo</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="1" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="1" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Dago</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Dago</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="1" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Presentación de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="1" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2691,98 +2823,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="1" t="n">
-        <v>46315</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr">
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Joan</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="1" t="n">
-        <v>46316</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Yunier</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="1" t="n">
-        <v>46317</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Dago</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr">
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="1" t="n">
-        <v>46321</v>
-      </c>
-      <c r="B90" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>46328</v>
+      </c>
+      <c r="B94" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2793,98 +2925,103 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Dago</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>46329</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Alana)
+11:00 - Github individual: Básicos</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="1" t="n">
-        <v>46322</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr"/>
-      <c r="D91" t="inlineStr">
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>46330</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Irene</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="1" t="n">
-        <v>46323</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Joan</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>46331</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="1" t="n">
-        <v>46324</v>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr">
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="1" t="n">
-        <v>46328</v>
-      </c>
-      <c r="B94" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>46335</v>
+      </c>
+      <c r="B98" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2895,98 +3032,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>46336</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="1" t="n">
-        <v>46329</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr">
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>46337</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Alana</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="1" t="n">
-        <v>46330</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Irene</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>46338</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="1" t="n">
-        <v>46331</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr">
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="1" t="n">
-        <v>46335</v>
-      </c>
-      <c r="B98" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="B102" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -2997,98 +3134,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>46343</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="1" t="n">
-        <v>46336</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr">
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>46344</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Dago</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="1" t="n">
-        <v>46337</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Alana</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>46345</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="1" t="n">
-        <v>46338</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr">
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="1" t="n">
-        <v>46342</v>
-      </c>
-      <c r="B102" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>46349</v>
+      </c>
+      <c r="B106" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3099,98 +3236,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>46350</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="1" t="n">
-        <v>46343</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr">
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>46351</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Yunier</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="1" t="n">
-        <v>46344</v>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Dago</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>46352</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="1" t="n">
-        <v>46345</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr">
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="1" t="n">
-        <v>46349</v>
-      </c>
-      <c r="B106" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>46356</v>
+      </c>
+      <c r="B110" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3201,98 +3338,98 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>46357</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="1" t="n">
-        <v>46350</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr">
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>46358</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Joan</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="1" t="n">
-        <v>46351</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Yunier</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>46359</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="1" t="n">
-        <v>46352</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Dago</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr">
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="1" t="n">
-        <v>46356</v>
-      </c>
-      <c r="B110" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>46370</v>
+      </c>
+      <c r="B114" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3303,98 +3440,103 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Dago</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>46371</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Alana)
+11:00 - De la Teoria a la Pràctica: Apps amb Streamlit</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="1" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr">
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>46372</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Irene</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="1" t="n">
-        <v>46358</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Joan</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>46373</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="1" t="n">
-        <v>46359</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr">
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="1" t="n">
-        <v>46370</v>
-      </c>
-      <c r="B114" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>46377</v>
+      </c>
+      <c r="B118" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3405,108 +3547,6 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Dago</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="1" t="n">
-        <v>46371</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr"/>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="1" t="n">
-        <v>46372</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Irene</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="1" t="n">
-        <v>46373</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>Presentación de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="1" t="n">
-        <v>46377</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Welcome: de 10:15 – 11:00 
-Weekly: 
-11:00 Alana 
-11:30 Joan 
-12:00 Yunier 
-12:30 Dago 
-13:00 Irene </t>
-        </is>
-      </c>
       <c r="D118" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-13 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -945,7 +945,11 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Tècniques  d'Anàlisi de dades en Customer Experience: NPS i CSAT</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>Dago</t>
@@ -1191,11 +1195,7 @@
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Yunier</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Yunier</t>
@@ -1217,7 +1217,11 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Yunier</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>Dago</t>
@@ -1274,7 +1278,7 @@
       <c r="C31" t="inlineStr">
         <is>
           <t>Píldora Aula Nucli
-11:00 - Buenas prácticas para dashboards</t>
+11:00 - Intro to Big Data with PySpark: A Hands-on Workshop with Real Booking.com Data</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1538,7 +1542,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Píldora Aula Nucli
+11:00 - Buenas prácticas para dashboards</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-15 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -887,9 +887,9 @@
       <c r="C17" t="inlineStr">
         <is>
           <t>Presentacions
-11:00 - Federico Urbina: TBD
-11:30 - Sabina Planas: TBD
-12:00 - Dioulde Diao: TBD</t>
+11:00 - Federico Urbina: Hacia una Barcelona Preventiva
+11:30 - Sabina Planas: From Diabetes Pills to Weight-Loss Medicines: How the Story of GLP-1 Drugs Changed in the Medical Literature
+12:00 - Dioulde Diao: Mapping cell-type-resolved transcriptional landscapes of primary and recurrent Glioblastoma at single-cell resolution</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -948,7 +948,7 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Dago)
-11:30 - Tècniques  d'Anàlisi de dades en Customer Experience: NPS i CSAT</t>
+11:30 - Tècniques  d'Anàlisi de dades en Customer Experience: NPS i CSAT amb R Program</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1543,12 +1543,7 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Píldora Aula Nucli
-11:00 - Buenas prácticas para dashboards</t>
-        </is>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -1815,7 +1810,7 @@
       <c r="C51" t="inlineStr">
         <is>
           <t>Píldora Aula Nucli
-11:00 - Un caso real de projecto en Booking.com</t>
+11:00 - Buenas prácticas para dashboards</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-27 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1107,7 +1107,6 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>Presentacions
-11:00 - Vanina Tonzo: TBD
 11:30 - Vanessa Bujaldon: TBD
 12:00 - Florencia Di Stefano: TBD</t>
         </is>
@@ -1447,7 +1446,8 @@
         <is>
           <t>Presentacions
 11:00 - Nakta Samipour: TBD
-11:30 - Raúl Martínez: TBD</t>
+11:30 - Raúl Martínez: TBD
+12:00 - Vanina Tonzo: TBD</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-28 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1107,8 +1107,8 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>Presentacions
-11:30 - Vanessa Bujaldon: TBD
-12:00 - Florencia Di Stefano: TBD</t>
+11:30 - Vanessa Bujaldon: Evaluating Digital Demand Signals and Territorial Mobility Patterns to Support Airline Seat Allocation
+12:00 - Jose Manuel Romero García: Análisis de los delitos de odio en la ciudad de Washington en el periodo 2012  - 2024</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1217,7 +1217,8 @@
       <c r="C29" t="inlineStr">
         <is>
           <t>Presentacions:
-11:00 - Elisa Volk: TBD</t>
+11:00 - Elisa Volk: TBD
+11:30 - Florencia Di Stefano: TBD</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-05-29 09:21
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1163,13 +1163,7 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Píldores Aula Nucli (Joan)
-10:00 - Introducció al Machine Learning (Supervisat vs No Supervisat)
-12:30 - Introducció al Network Analysis (Graph Theory)</t>
-        </is>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Joan</t>
@@ -1447,7 +1441,8 @@
           <t>Presentacions
 11:00 - Nakta Samipour: TBD
 11:30 - Raúl Martínez: TBD
-12:00 - Vanina Tonzo: TBD</t>
+12:00 - Vanina Tonzo: TBD
+12:30 - Vanessa Bujaldon: Evaluating Digital Demand Signals and Territorial Mobility Patterns to Support Airline Seat Allocation</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1714,8 +1709,8 @@
       <c r="C47" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Joan)
-10:00 - Workshop Machine Learning No Supervisat (Clustering, PCA i Outlier Detection)
-12:30 - Workshop Machine Learning Supervisat (Random Forest)</t>
+10:00 - Introducció al Machine Learning (Supervisat vs No Supervisat)
+12:30 - Introducció al Network Analysis (Graph Theory)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2239,7 +2234,13 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Joan)
+10:00 - Workshop Machine Learning No Supervisat (Clustering, PCA i Outlier Detection)
+12:30 - Workshop Machine Learning Supervisat (Random Forest)</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
           <t>Joan</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-03 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1209,9 +1209,10 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Presentacions:
-11:00 - Elisa Volk: TBD
-11:30 - Florencia Di Stefano: TBD</t>
+          <t xml:space="preserve">Presentacions:
+11:00 - Giorgia Calvagna: The Protein Shift
+11:30 - Florencia Di Stefano: Política con perspectiva de género: Monitoreo de la participación política de mujeres y diversidades en Argentina
+</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1325,7 +1326,7 @@
       <c r="C33" t="inlineStr">
         <is>
           <t>Presentacions:
-11:00 - Giorgia Calvagna: TBD
+11:00 - Elisa Volk: Beyond the binary: Understanding Toxicity and Hate Speech Patterns Across Online Communities
 11:30 - Jordi Lamarca: TBD</t>
         </is>
       </c>
@@ -1441,7 +1442,6 @@
           <t>Presentacions
 11:00 - Nakta Samipour: TBD
 11:30 - Raúl Martínez: TBD
-12:00 - Vanina Tonzo: TBD
 12:30 - Vanessa Bujaldon: Evaluating Digital Demand Signals and Territorial Mobility Patterns to Support Airline Seat Allocation</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-09 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1300,7 +1300,8 @@
         <is>
           <t>Incubadora de Projectes amb Joan
 Presentacions:
-11:00 - Didac Petit: TBD</t>
+11:00 - Didac Petit: Anàlisi de les característiques tecnicobiomecàniques del calçat de trail running 
+en funció del perfil del corredor</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1328,7 +1329,7 @@
         <is>
           <t>Presentacions:
 11:00 - Elisa Volk: Beyond the binary: Understanding Toxicity and Hate Speech Patterns Across Online Communities
-11:30 - Jordi Lamarca: TBD</t>
+11:30 - Jordi Lamarca: Overtake.gp: data analytics d'un mitjà digital a 200 km/h</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-11 09:57
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1329,7 +1329,9 @@
         <is>
           <t>Presentacions:
 11:00 - Elisa Volk: Beyond the binary: Understanding Toxicity and Hate Speech Patterns Across Online Communities
-11:30 - Jordi Lamarca: Overtake.gp: data analytics d'un mitjà digital a 200 km/h</t>
+11:30 - Jordi Lamarca: Overtake.gp: data analytics d'un mitjà digital a 200 km/h
+12:00 - Emmanuel Gonzalez Moreno: ¿QUIÉN TIENE TIEMPO LIBRE EN CATALUÑA? UN ANÁLISIS DE LAS DESIGUALDADES TEMPORALES SEGÚN GÉNERO, CICLO VITAL Y SITUACIÓN LABORAL A PARTIR DE LA ENCUESTA DE USO DEL TIEMPO 2024
+12:30 - Santiago Alvarez Salvado: Criminalidad en Cataluña: anatomía de lo que dicen (y callan) los datos</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-16 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1443,10 +1443,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Presentacions
-11:00 - Nakta Samipour: TBD
-11:30 - Raúl Martínez: TBD
-12:30 - Vanessa Bujaldon: Evaluating Digital Demand Signals and Territorial Mobility Patterns to Support Airline Seat Allocation</t>
+          <t xml:space="preserve">Presentacions
+11:30 - Vanessa Bujaldon: Evaluating Digital Demand Signals and Territorial Mobility Patterns to Support Airline Seat Allocation
+12:00 - Nakta Samipour: TBD
+12:30 - Raúl Martínez: TBD
+</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-19 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1444,8 +1444,11 @@
       <c r="C37" t="inlineStr">
         <is>
           <t xml:space="preserve">Presentacions
+10:00- Nizar -&gt; Com una biblioteca corba l'espai-temps: la performance de la Xarxa de Biblioteques de la ciutat de Barcelona
+10:30 - Roger -&gt; GO / NO GO - Intelligent Sea Breeze Prediction System for Water Sports Using Machine Learning
+11:00 - Hamza -&gt; ¿Están disminuyendo las abejas? Análisis del impacto agrícola y climático sobre las colmenas
 11:30 - Vanessa Bujaldon: Evaluating Digital Demand Signals and Territorial Mobility Patterns to Support Airline Seat Allocation
-12:00 - Nakta Samipour: TBD
+12:00 - Nakta Samipour: Sustainable e-commerce route planning
 12:30 - Raúl Martínez: Diario de Catalunya. Una sociedad en el tiempo
 </t>
         </is>
@@ -1555,7 +1558,13 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presentacions
+11:00 - Sara Ossa: ¿Llegan las ayudas a la compra donde más se necesitan? Análisis de accesibilidad y política pública en España
+</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -1848,7 +1857,8 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Joan</t>
+          <t>Reservat dinàmica Eli. Horari 11:00-13:00
+Incubadora Projectes (Joan): 10:00-11:00 // 13:00-14:00</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1929,7 +1939,8 @@
       <c r="C55" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Alana)
-11:00 - Github en equipo: Básicos</t>
+10:00 - Github en equipo: Básicos
+12:00 - Reservat dinàmica Eli</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-29 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1619,7 +1619,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Yunier)
+11:30 - Introducción de Redes Neuronales</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-06-30 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1998,7 +1998,14 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Presentacions Finals
+11:00 - Marta Torrente: TBD
+11:30 - Iván Joseph Aguilar: TBD
+12:00 - Mani Rezaeirad: TBD</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>Joan</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-02 09:21
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1269,12 +1269,7 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Píldora Aula Nucli
-11:00 - Intro to Big Data with PySpark: A Hands-on Workshop with Real Booking.com Data</t>
-        </is>
-      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -1672,7 +1667,11 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>11:00 Marcos Molina Martínez: Revolución analítica en la NBA (2000–2025): transformación de las zonas de lanzamiento e impacto en el rendimiento deportivo y económico.</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>Alana</t>
@@ -1837,7 +1836,7 @@
       <c r="C51" t="inlineStr">
         <is>
           <t>Píldora Aula Nucli
-11:00 - Buenas prácticas para dashboards</t>
+11:00 - Intro to Big Data with PySpark: A Hands-on Workshop with Booking.com Data</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2003,7 +2002,8 @@
           <t>Presentacions Finals
 11:00 - Marta Torrente: TBD
 11:30 - Iván Joseph Aguilar: TBD
-12:00 - Mani Rezaeirad: TBD</t>
+12:00 - Mani Rezaeirad: TBD
+12:30 - Héctor Morales: TBD</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-07 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1944,8 +1944,8 @@
       <c r="C55" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Alana)
-10:00 - Github en equipo: Básicos
-12:00 - Reservat dinàmica Eli</t>
+10:00 - ¿Sobrevivirías al Titanic? Clasificación supervisada con Machine Learning
+12:00 - Reservat dinàmica Elixabete</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2000,6 +2000,7 @@
       <c r="C57" t="inlineStr">
         <is>
           <t>Presentacions Finals
+10:30 - Gledson Jardim de Vargas: TBD
 11:00 - Marta Torrente: TBD
 11:30 - Iván Joseph Aguilar: TBD
 12:00 - Mani Rezaeirad: TBD
@@ -2059,7 +2060,11 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Análisis de Sentimientos para Estrategias de Marketing en R: Caso Zapatillas Nike</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>Dago</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-08 09:23
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1728,7 +1728,7 @@
       <c r="C47" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Joan)
-10:00 - Introducció al Machine Learning (Supervisat vs No Supervisat)
+10:40 - Introducció al Machine Learning (Supervisat vs No Supervisat)
 12:30 - Introducció al Network Analysis (Graph Theory)</t>
         </is>
       </c>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Datathon estiuenc
+          <t>Datathon estiuenc 10.30
 Aula Principal
 Activitat en grups "competitiva", base de dades de viatges d'estiu</t>
         </is>
@@ -2004,7 +2004,8 @@
 11:00 - Marta Torrente: TBD
 11:30 - Iván Joseph Aguilar: TBD
 12:00 - Mani Rezaeirad: TBD
-12:30 - Héctor Morales: TBD</t>
+12:30 - Héctor Morales: TBD
+14:00 ""Networking"" 😉</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-08 09:38
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1862,7 +1862,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Reservat dinàmica Eli. Horari 11:00-13:00
+          <t>11:00-13:00. Gestió de l'estrés. Eli.
 Incubadora Projectes (Joan): 10:00-11:00 // 13:00-14:00</t>
         </is>
       </c>
@@ -1945,7 +1945,7 @@
         <is>
           <t>Píldores Aula Nucli (Alana)
 10:00 - ¿Sobrevivirías al Titanic? Clasificación supervisada con Machine Learning
-12:00 - Reservat dinàmica Elixabete</t>
+12:00-14:00. Gestió del temps. Eli.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-10 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1944,7 +1944,7 @@
       <c r="C55" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Alana)
-10:00 - ¿Sobrevivirías al Titanic? Clasificación supervisada con Machine Learning
+10:00 - 12:00 ¿Sobrevivirías al Titanic? Clasificación supervisada con Machine Learning
 12:00-14:00. Gestió del temps. Eli.</t>
         </is>
       </c>
@@ -2005,6 +2005,7 @@
 11:30 - Iván Joseph Aguilar: TBD
 12:00 - Mani Rezaeirad: TBD
 12:30 - Héctor Morales: TBD
+13:00 - Michela Vistarini: TBD
 14:00 ""Networking"" 😉</t>
         </is>
       </c>
@@ -2113,7 +2114,16 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presentacions Finals
+10:30 - Ana Ibáñez: TBD
+11:00 - Mariela Villca Vizalla: TBD
+11:30 - Tania Esther Adrianzen Acero: TBD
+12:00 - Ángel Herrezuelo Hernández: TBD
+</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-14 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1803,6 +1803,115 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
+          <t xml:space="preserve">
+Weekly: 
+11:00 Alana 
+11:30 Joan 
+12:00 Yunier 
+12:30 Dago 
+13:00 Irene </t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Welcome: de 10:15 – 11:00 
+Píldora Aula Nucli
+11:00 - Intro to Big Data with PySpark: A Hands-on Workshop with Booking.com Data</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>11:00-13:00. Gestió de l'estrés. Eli.
+Incubadora Projectes (Joan): 10:00-11:00 // 13:00-14:00</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Presentación de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
 11:00 Alana 
@@ -1812,114 +1921,6 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>46217</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Píldora Aula Nucli
-11:00 - Intro to Big Data with PySpark: A Hands-on Workshop with Booking.com Data</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>46218</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>11:00-13:00. Gestió de l'estrés. Eli.
-Incubadora Projectes (Joan): 10:00-11:00 // 13:00-14:00</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>46219</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Presentación de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>46223</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Welcome: de 10:15 – 11:00 
-Weekly: 
-11:00 Alana 
-11:30 Joan 
-12:00 Yunier 
-12:30 Dago 
-13:00 Irene </t>
-        </is>
-      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>Dago</t>
@@ -1971,7 +1972,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Datathon estiuenc 10.30
+          <t>Datathon estiuenc 10.15
 Aula Principal
 Activitat en grups "competitiva", base de dades de viatges d'estiu</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-16 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1888,7 +1888,11 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>12:00 Jaume Rafols: Anàlisi del finançament de les administracions públiques de Catalunya als mitjans de comunicació (2015-2024)</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-21 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1890,7 +1890,8 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>12:00 Jaume Rafols: Anàlisi del finançament de les administracions públiques de Catalunya als mitjans de comunicació (2015-2024)</t>
+          <t>Presentacions Finals
+12:00 Jaume Rafols: Anàlisi del finançament de les administracions públiques de Catalunya als mitjans de comunicació (2015-2024)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2010,7 +2011,7 @@
 11:30 - Iván Joseph Aguilar: TBD
 12:00 - Mani Rezaeirad: Early Anticipation for Extended ICU Stays in Lung Cancer Patients
 12:30 - Héctor Morales: TBD
-13:00 - Michela Vistarini: TBD
+13:00 - Michela Vistarini: Vulnerabilitat climàtica i cobertura de la xarxa de refugis a Barcelona: una anàlisi d'equitat a escala de barri
 14:00 ""Networking"" 😉</t>
         </is>
       </c>
@@ -2121,12 +2122,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presentacions Finals
+          <t>Presentacions Finals
 10:30 - Ana Ibáñez: TBD
 11:00 - Mariela Villca Vizalla: TBD
 11:30 - Tania Esther Adrianzen Acero: TBD
 12:00 - Ángel Herrezuelo Hernández: TBD
-</t>
+12:30 - Jordi Calmet: TBD</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-22 09:31
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -1977,7 +1977,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Datathon estiuenc 10.15
+          <t>Datathon estiuenc 10.30
 Aula Principal
 Activitat en grups "competitiva", base de dades de viatges d'estiu</t>
         </is>
@@ -2007,11 +2007,10 @@
         <is>
           <t>Presentacions Finals
 10:30 - Gledson Jardim de Vargas: TBD
-11:00 - Marta Torrente: TBD
-11:30 - Iván Joseph Aguilar: TBD
-12:00 - Mani Rezaeirad: Early Anticipation for Extended ICU Stays in Lung Cancer Patients
-12:30 - Héctor Morales: TBD
-13:00 - Michela Vistarini: Vulnerabilitat climàtica i cobertura de la xarxa de refugis a Barcelona: una anàlisi d'equitat a escala de barri
+11:00 - Marta Torrente: People Analytics: Un framework para la evaluación del bienestar laboral y la cultura organizacional
+11:30 - Mani Rezaeirad: Early Anticipation for Extended ICU Stays in Lung Cancer Patients
+12:00 - Héctor Morales: TBD
+12:30 - Michela Vistarini: Vulnerabilitat climàtica i cobertura de la xarxa de refugis a Barcelona: una anàlisi d'equitat a escala de barri
 14:00 ""Networking"" 😉</t>
         </is>
       </c>
@@ -2127,7 +2126,8 @@
 11:00 - Mariela Villca Vizalla: TBD
 11:30 - Tania Esther Adrianzen Acero: TBD
 12:00 - Ángel Herrezuelo Hernández: TBD
-12:30 - Jordi Calmet: TBD</t>
+12:30 - Jordi Calmet: TBD
+13:00 - Iván Joseph Aguilar Monteza: TBD</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-28 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2070,7 +2070,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Análisis de Sentimientos para Estrategias de Marketing en R: Caso Zapatillas Nike</t>
+          <t>11:30 Análisis de Sentimientos para Estrategias de Marketing en R: Caso Zapatillas Nike</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2096,7 +2096,10 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Alana</t>
+          <t>Incubadora de Projectes amb Alana
+Presentacions Finals
+11:00 - Ángel Herrezuelo Hernández: Delitos de odio y discurso público en España
+11:30 - Ana Ibáñez: Asentamientos de colonos en Cisjordania: expansión territorial, población y violencia</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2123,10 +2126,9 @@
       <c r="C61" t="inlineStr">
         <is>
           <t>Presentacions Finals
-10:30 - Ana Ibáñez: TBD
 11:00 - Mariela Villca Vizalla: TBD
-11:30 - Tania Esther Adrianzen Acero: TBD
-12:00 - Ángel Herrezuelo Hernández: TBD
+11:30 - Tania Esther Adrianzen Acero: La presencia latinoamericana en el cine español. Una aproximación desde los ámbitos de producción, guión y dirección.
+12:00 - 
 12:30 - Jordi Calmet: TBD
 13:00 - Iván Joseph Aguilar Monteza: TBD</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-29 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2070,7 +2070,8 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>11:30 Análisis de Sentimientos para Estrategias de Marketing en R: Caso Zapatillas Nike</t>
+          <t xml:space="preserve">11:30 Análisis de Sentimientos para Estrategias de Marketing en R: Caso Zapatillas Nike
+</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2098,8 +2099,10 @@
         <is>
           <t>Incubadora de Projectes amb Alana
 Presentacions Finals
+10:30 Marius-Asociación entre Actividad Física y Síntomas Depresivos
 11:00 - Ángel Herrezuelo Hernández: Delitos de odio y discurso público en España
-11:30 - Ana Ibáñez: Asentamientos de colonos en Cisjordania: expansión territorial, población y violencia</t>
+11:30 - Ana Ibáñez: Asentamientos de colonos en Cisjordania: expansión territorial, población y violencia
+12:00 - Jordi Calmet: Canciones en la pantalla: ¿grandes films, grandes hits?</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2123,16 +2126,7 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Presentacions Finals
-11:00 - Mariela Villca Vizalla: TBD
-11:30 - Tania Esther Adrianzen Acero: La presencia latinoamericana en el cine español. Una aproximación desde los ámbitos de producción, guión y dirección.
-12:00 - 
-12:30 - Jordi Calmet: TBD
-13:00 - Iván Joseph Aguilar Monteza: TBD</t>
-        </is>
-      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-07-29 14:01
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2070,8 +2070,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">11:30 Análisis de Sentimientos para Estrategias de Marketing en R: Caso Zapatillas Nike
-</t>
+          <t>11:30 Análisis de Sentimientos para Estrategias de Marketing en R: Caso Zapatillas Nike</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2101,8 +2100,7 @@
 Presentacions Finals
 10:30 Marius-Asociación entre Actividad Física y Síntomas Depresivos
 11:00 - Ángel Herrezuelo Hernández: Delitos de odio y discurso público en España
-11:30 - Ana Ibáñez: Asentamientos de colonos en Cisjordania: expansión territorial, población y violencia
-12:00 - Jordi Calmet: Canciones en la pantalla: ¿grandes films, grandes hits?</t>
+11:30 - Ana Ibáñez: Asentamientos de colonos en Cisjordania: expansión territorial, población y violencia</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2126,7 +2124,19 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Presentacions Finals
+10:00 Valeria - Neural Network Classification of Alzheimer's Disease from Brain MRI Images
+10:30 : Fiametta - Patrones de las Fake News
+11:00 - Mariela Villca Vizalla: TBD
+11:30 - Tania Esther Adrianzen Acero: La presencia latinoamericana en el cine español. Una aproximación desde los ámbitos de producción, guión y dirección.
+12:00 - Macarena: De la protesta a la transición: minería de textos y análisis del discurso en la cobertura de El País sobre la Revolución Tunecina
+12:30 - Jordi Calmet: TBD
+13:00 - Iván Joseph Aguilar Monteza: TBD
+13:30-Alejandro - Asociación entre la duración del sueño y las características demográficas, los indicadores de salud y los factores del estilo de vida.</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-08-03 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2237,7 +2237,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Presentacions Finals
+11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr">
         <is>
           <t>Alana</t>
@@ -2508,10 +2513,8 @@
       <c r="C75" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Alana)
-Todo Python
-10:30 - Estructuras de datos
-11:30 - Estructuras de control
-12:30 - Funciones</t>
+Dinámica Grupal
+11:00 MVP: Producto mínimo viable</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">

</xml_diff>